<commit_message>
feat: Add settings page for managing BBM prices, vehicles, and drivers
- Implemented a new settings page to manage BBM prices, vehicles, and drivers.
- Added functionality to add, edit, and delete BBM prices.
- Enabled management of vehicles and their associated drivers and BBM types.
- Introduced autofill feature for BBM type and driver based on selected vehicle.
- Updated PDF generation to reflect changes in BBM prices and vehicle data.
- Enhanced user interface with new styles for settings management.
</commit_message>
<xml_diff>
--- a/exports/data-bon-bbm.xlsx
+++ b/exports/data-bon-bbm.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Rekap Bon BBM" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Agustus 2026" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="September 2026" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Oktober 2026" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Bon BBM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agustus 2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="September 2026" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oktober 2026" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Rekap Bon BBM'!$A$1:$H$10</definedName>
@@ -1398,7 +1398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="2"/>
@@ -2061,34 +2061,118 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="13" t="n"/>
-      <c r="E18" s="13" t="n"/>
-      <c r="F18" s="12" t="n"/>
-      <c r="G18" s="12" t="n"/>
-      <c r="H18" s="12" t="n"/>
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>H 123 H</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Pertamax</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>11111</v>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>Sebelas Ribu Seratus Sebelas Rupiah</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>BOWO</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 10:07:10</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n"/>
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="13" t="n"/>
-      <c r="E19" s="13" t="n"/>
-      <c r="F19" s="12" t="n"/>
-      <c r="G19" s="12" t="n"/>
-      <c r="H19" s="12" t="n"/>
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>H 1275 XR</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Pertamax</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>Dua Ratus Ribu Rupiah</t>
+        </is>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>WANDI</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:25:21</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="13" t="n"/>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="12" t="n"/>
-      <c r="G20" s="12" t="n"/>
-      <c r="H20" s="12" t="n"/>
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>H 1275 XR</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>Pertamax</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>18.81</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>300000</v>
+      </c>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>Tiga Ratus Ribu Rupiah</t>
+        </is>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>WANDI</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:26:25</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
@@ -2429,6 +2513,196 @@
       <c r="H29" s="12" t="inlineStr">
         <is>
           <t>2026-09-09 09:28:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>B 1924 KJA</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Pertamina Dex</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>19.84</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>Lima Ratus Ribu Rupiah</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>SATRIA</t>
+        </is>
+      </c>
+      <c r="H30" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:28:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>H 1275 XR</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Pertamax</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>Dua Ratus Ribu Rupiah</t>
+        </is>
+      </c>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>WANDI</t>
+        </is>
+      </c>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:30:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>H 1142 XG</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Pertamax</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>25.08</v>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>400000</v>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>Empat Ratus Ribu Rupiah</t>
+        </is>
+      </c>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>ANDRI</t>
+        </is>
+      </c>
+      <c r="H32" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:31:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>H 1715 XR</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Pertamax</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>18.81</v>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>300000</v>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>Tiga Ratus Ribu Rupiah</t>
+        </is>
+      </c>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>LUKMAN</t>
+        </is>
+      </c>
+      <c r="H33" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:32:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>H 1274 XR</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>Pertamax</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>159500</v>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>Seratus Lima Puluh Sembilan Ribu Lima Ratus Rupiah</t>
+        </is>
+      </c>
+      <c r="G34" s="14" t="inlineStr">
+        <is>
+          <t>YULI</t>
+        </is>
+      </c>
+      <c r="H34" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:38:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
.git/COMMIT_EDITMSG [unix] (15:24 10/09/2026)                                                                                                   1,1 Top "~/Downloads/simbon-bbm/simbon-bbm/.git/COMMIT_EDITMSG" [unix] 54L, 2043Bfeat: Add settings page for managing BBM prices, vehicles, and drivers
- Implemented a new settings page to manage BBM prices, vehicles, and drivers.
- Added functionality to add, edit, and delete BBM prices.
- Enabled management of vehicles and their associated drivers and BBM types.
- Introduced autofill feature for BBM type and driver based on selected vehicle.
- Updated PDF generation to reflect changes in BBM prices and vehicle data.
- Enhanced user interface with new styles for settings management.
</commit_message>
<xml_diff>
--- a/exports/data-bon-bbm.xlsx
+++ b/exports/data-bon-bbm.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Rekap Bon BBM" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Agustus 2026" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="September 2026" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Oktober 2026" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Bon BBM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agustus 2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="September 2026" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oktober 2026" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Rekap Bon BBM'!$A$1:$H$10</definedName>
@@ -1398,7 +1398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="2"/>
@@ -2061,34 +2061,118 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="13" t="n"/>
-      <c r="E18" s="13" t="n"/>
-      <c r="F18" s="12" t="n"/>
-      <c r="G18" s="12" t="n"/>
-      <c r="H18" s="12" t="n"/>
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>H 123 H</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Pertamax</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>11111</v>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>Sebelas Ribu Seratus Sebelas Rupiah</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>BOWO</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 10:07:10</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n"/>
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="13" t="n"/>
-      <c r="E19" s="13" t="n"/>
-      <c r="F19" s="12" t="n"/>
-      <c r="G19" s="12" t="n"/>
-      <c r="H19" s="12" t="n"/>
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>H 1275 XR</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Pertamax</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>Dua Ratus Ribu Rupiah</t>
+        </is>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>WANDI</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:25:21</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="13" t="n"/>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="12" t="n"/>
-      <c r="G20" s="12" t="n"/>
-      <c r="H20" s="12" t="n"/>
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>H 1275 XR</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>Pertamax</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>18.81</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>300000</v>
+      </c>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>Tiga Ratus Ribu Rupiah</t>
+        </is>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>WANDI</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:26:25</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
@@ -2429,6 +2513,196 @@
       <c r="H29" s="12" t="inlineStr">
         <is>
           <t>2026-09-09 09:28:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>B 1924 KJA</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Pertamina Dex</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>19.84</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>Lima Ratus Ribu Rupiah</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>SATRIA</t>
+        </is>
+      </c>
+      <c r="H30" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:28:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>H 1275 XR</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Pertamax</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>Dua Ratus Ribu Rupiah</t>
+        </is>
+      </c>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>WANDI</t>
+        </is>
+      </c>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:30:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>H 1142 XG</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Pertamax</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>25.08</v>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>400000</v>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>Empat Ratus Ribu Rupiah</t>
+        </is>
+      </c>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>ANDRI</t>
+        </is>
+      </c>
+      <c r="H32" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:31:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>H 1715 XR</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Pertamax</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>18.81</v>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>300000</v>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>Tiga Ratus Ribu Rupiah</t>
+        </is>
+      </c>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>LUKMAN</t>
+        </is>
+      </c>
+      <c r="H33" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:32:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>H 1274 XR</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>Pertamax</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>159500</v>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>Seratus Lima Puluh Sembilan Ribu Lima Ratus Rupiah</t>
+        </is>
+      </c>
+      <c r="G34" s="14" t="inlineStr">
+        <is>
+          <t>YULI</t>
+        </is>
+      </c>
+      <c r="H34" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:38:20</t>
         </is>
       </c>
     </row>

</xml_diff>